<commit_message>
Add tourist-revenue sheet (3 provinces, 2023-2026) to Arrival province file
</commit_message>
<xml_diff>
--- a/output/Arrival province 2019-2026.xlsx
+++ b/output/Arrival province 2019-2026.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue from tourists" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -88,6 +90,9 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -143,7 +148,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -196,6 +201,9 @@
     <xf numFmtId="164" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3575,4 +3583,2456 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Revenue from tourists (รายได้จากผู้เยี่ยมเยือน) — Unit: Million THB</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sources: MOTS provincial files (2567 full year R; 2569 Jan-Jun, Apr-Jun preliminary; 2023/2025 from comparison columns). Domestics = คนไทย, International = ชาวต่างชาติ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="18" t="inlineStr">
+        <is>
+          <t>Bangkok — Revenue (M THB)</t>
+        </is>
+      </c>
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5">
+        <f>SUM(B6:B7)</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>SUM(C6:C7)</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>SUM(D6:D7)</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>SUM(E6:E7)</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>SUM(F6:F7)</f>
+        <v/>
+      </c>
+      <c r="G5">
+        <f>SUM(G6:G7)</f>
+        <v/>
+      </c>
+      <c r="H5">
+        <f>SUM(H6:H7)</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>SUM(I6:I7)</f>
+        <v/>
+      </c>
+      <c r="J5">
+        <f>SUM(J6:J7)</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>SUM(K6:K7)</f>
+        <v/>
+      </c>
+      <c r="L5">
+        <f>SUM(L6:L7)</f>
+        <v/>
+      </c>
+      <c r="M5">
+        <f>SUM(M6:M7)</f>
+        <v/>
+      </c>
+      <c r="N5">
+        <f>SUM(B5:M5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15770.84</v>
+      </c>
+      <c r="C6" t="n">
+        <v>14466.82</v>
+      </c>
+      <c r="D6" t="n">
+        <v>17809.1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>26871.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>26999.5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>23575</v>
+      </c>
+      <c r="H6" t="n">
+        <v>19847.97</v>
+      </c>
+      <c r="I6" t="n">
+        <v>23941.35</v>
+      </c>
+      <c r="J6" t="n">
+        <v>24644.66</v>
+      </c>
+      <c r="K6" t="n">
+        <v>20052.22</v>
+      </c>
+      <c r="L6" t="n">
+        <v>23663.02</v>
+      </c>
+      <c r="M6" t="n">
+        <v>23040.8</v>
+      </c>
+      <c r="N6">
+        <f>SUM(B6:M6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>46497.38</v>
+      </c>
+      <c r="C7" t="n">
+        <v>46626.39</v>
+      </c>
+      <c r="D7" t="n">
+        <v>49176.34</v>
+      </c>
+      <c r="E7" t="n">
+        <v>45017.35</v>
+      </c>
+      <c r="F7" t="n">
+        <v>42251.74</v>
+      </c>
+      <c r="G7" t="n">
+        <v>47027.65</v>
+      </c>
+      <c r="H7" t="n">
+        <v>54316.54</v>
+      </c>
+      <c r="I7" t="n">
+        <v>53747.62</v>
+      </c>
+      <c r="J7" t="n">
+        <v>47174.66</v>
+      </c>
+      <c r="K7" t="n">
+        <v>49288.24</v>
+      </c>
+      <c r="L7" t="n">
+        <v>54084.57</v>
+      </c>
+      <c r="M7" t="n">
+        <v>60412.81</v>
+      </c>
+      <c r="N7">
+        <f>SUM(B7:M7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B8" s="19">
+        <f>B6/B5</f>
+        <v/>
+      </c>
+      <c r="C8" s="19">
+        <f>C6/C5</f>
+        <v/>
+      </c>
+      <c r="D8" s="19">
+        <f>D6/D5</f>
+        <v/>
+      </c>
+      <c r="E8" s="19">
+        <f>E6/E5</f>
+        <v/>
+      </c>
+      <c r="F8" s="19">
+        <f>F6/F5</f>
+        <v/>
+      </c>
+      <c r="G8" s="19">
+        <f>G6/G5</f>
+        <v/>
+      </c>
+      <c r="H8" s="19">
+        <f>H6/H5</f>
+        <v/>
+      </c>
+      <c r="I8" s="19">
+        <f>I6/I5</f>
+        <v/>
+      </c>
+      <c r="J8" s="19">
+        <f>J6/J5</f>
+        <v/>
+      </c>
+      <c r="K8" s="19">
+        <f>K6/K5</f>
+        <v/>
+      </c>
+      <c r="L8" s="19">
+        <f>L6/L5</f>
+        <v/>
+      </c>
+      <c r="M8" s="19">
+        <f>M6/M5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B9">
+        <f>SUM(B10:B11)</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>SUM(C10:C11)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>SUM(D10:D11)</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>SUM(E10:E11)</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>SUM(F10:F11)</f>
+        <v/>
+      </c>
+      <c r="G9">
+        <f>SUM(G10:G11)</f>
+        <v/>
+      </c>
+      <c r="H9">
+        <f>SUM(H10:H11)</f>
+        <v/>
+      </c>
+      <c r="I9">
+        <f>SUM(I10:I11)</f>
+        <v/>
+      </c>
+      <c r="J9">
+        <f>SUM(J10:J11)</f>
+        <v/>
+      </c>
+      <c r="K9">
+        <f>SUM(K10:K11)</f>
+        <v/>
+      </c>
+      <c r="L9">
+        <f>SUM(L10:L11)</f>
+        <v/>
+      </c>
+      <c r="M9">
+        <f>SUM(M10:M11)</f>
+        <v/>
+      </c>
+      <c r="N9">
+        <f>SUM(B9:M9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>17970.96</v>
+      </c>
+      <c r="C10" t="n">
+        <v>14875.52</v>
+      </c>
+      <c r="D10" t="n">
+        <v>15796.22</v>
+      </c>
+      <c r="E10" t="n">
+        <v>26385.77</v>
+      </c>
+      <c r="F10" t="n">
+        <v>26283.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>23157.58</v>
+      </c>
+      <c r="H10" t="n">
+        <v>21284.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>25665.4</v>
+      </c>
+      <c r="J10" t="n">
+        <v>25871.12</v>
+      </c>
+      <c r="K10" t="n">
+        <v>26334.91</v>
+      </c>
+      <c r="L10" t="n">
+        <v>22288.42</v>
+      </c>
+      <c r="M10" t="n">
+        <v>26376.43</v>
+      </c>
+      <c r="N10">
+        <f>SUM(B10:M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>58366.84</v>
+      </c>
+      <c r="C11" t="n">
+        <v>60814.75</v>
+      </c>
+      <c r="D11" t="n">
+        <v>53833.56</v>
+      </c>
+      <c r="E11" t="n">
+        <v>51705.81</v>
+      </c>
+      <c r="F11" t="n">
+        <v>49153.21</v>
+      </c>
+      <c r="G11" t="n">
+        <v>52208.26</v>
+      </c>
+      <c r="H11" t="n">
+        <v>54942.64</v>
+      </c>
+      <c r="I11" t="n">
+        <v>53888.28</v>
+      </c>
+      <c r="J11" t="n">
+        <v>47296.28</v>
+      </c>
+      <c r="K11" t="n">
+        <v>56541.99</v>
+      </c>
+      <c r="L11" t="n">
+        <v>62565.7</v>
+      </c>
+      <c r="M11" t="n">
+        <v>68585.09</v>
+      </c>
+      <c r="N11">
+        <f>SUM(B11:M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B12" s="19">
+        <f>B10/B9</f>
+        <v/>
+      </c>
+      <c r="C12" s="19">
+        <f>C10/C9</f>
+        <v/>
+      </c>
+      <c r="D12" s="19">
+        <f>D10/D9</f>
+        <v/>
+      </c>
+      <c r="E12" s="19">
+        <f>E10/E9</f>
+        <v/>
+      </c>
+      <c r="F12" s="19">
+        <f>F10/F9</f>
+        <v/>
+      </c>
+      <c r="G12" s="19">
+        <f>G10/G9</f>
+        <v/>
+      </c>
+      <c r="H12" s="19">
+        <f>H10/H9</f>
+        <v/>
+      </c>
+      <c r="I12" s="19">
+        <f>I10/I9</f>
+        <v/>
+      </c>
+      <c r="J12" s="19">
+        <f>J10/J9</f>
+        <v/>
+      </c>
+      <c r="K12" s="19">
+        <f>K10/K9</f>
+        <v/>
+      </c>
+      <c r="L12" s="19">
+        <f>L10/L9</f>
+        <v/>
+      </c>
+      <c r="M12" s="19">
+        <f>M10/M9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="18" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13">
+        <f>SUM(B14:B15)</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>SUM(C14:C15)</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>SUM(D14:D15)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUM(E14:E15)</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>SUM(F14:F15)</f>
+        <v/>
+      </c>
+      <c r="G13">
+        <f>SUM(G14:G15)</f>
+        <v/>
+      </c>
+      <c r="H13">
+        <f>SUM(H14:H15)</f>
+        <v/>
+      </c>
+      <c r="I13">
+        <f>SUM(I14:I15)</f>
+        <v/>
+      </c>
+      <c r="J13">
+        <f>SUM(J14:J15)</f>
+        <v/>
+      </c>
+      <c r="K13">
+        <f>SUM(K14:K15)</f>
+        <v/>
+      </c>
+      <c r="L13">
+        <f>SUM(L14:L15)</f>
+        <v/>
+      </c>
+      <c r="M13">
+        <f>SUM(M14:M15)</f>
+        <v/>
+      </c>
+      <c r="N13">
+        <f>SUM(B13:M13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>14785.79</v>
+      </c>
+      <c r="C14" t="n">
+        <v>16307.35</v>
+      </c>
+      <c r="D14" t="n">
+        <v>18165.02</v>
+      </c>
+      <c r="E14" t="n">
+        <v>23281.21</v>
+      </c>
+      <c r="F14" t="n">
+        <v>26280.24</v>
+      </c>
+      <c r="G14" t="n">
+        <v>23555.64</v>
+      </c>
+      <c r="N14">
+        <f>SUM(B14:M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>65742.49000000001</v>
+      </c>
+      <c r="C15" t="n">
+        <v>56988.07</v>
+      </c>
+      <c r="D15" t="n">
+        <v>49844.62</v>
+      </c>
+      <c r="E15" t="n">
+        <v>46536.51</v>
+      </c>
+      <c r="F15" t="n">
+        <v>41885.47</v>
+      </c>
+      <c r="G15" t="n">
+        <v>42967.27</v>
+      </c>
+      <c r="N15">
+        <f>SUM(B15:M15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B16" s="19">
+        <f>B14/B13</f>
+        <v/>
+      </c>
+      <c r="C16" s="19">
+        <f>C14/C13</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>D14/D13</f>
+        <v/>
+      </c>
+      <c r="E16" s="19">
+        <f>E14/E13</f>
+        <v/>
+      </c>
+      <c r="F16" s="19">
+        <f>F14/F13</f>
+        <v/>
+      </c>
+      <c r="G16" s="19">
+        <f>G14/G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B17">
+        <f>SUM(B18:B19)</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>SUM(C18:C19)</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>SUM(D18:D19)</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>SUM(E18:E19)</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>SUM(F18:F19)</f>
+        <v/>
+      </c>
+      <c r="G17">
+        <f>SUM(G18:G19)</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>SUM(H18:H19)</f>
+        <v/>
+      </c>
+      <c r="I17">
+        <f>SUM(I18:I19)</f>
+        <v/>
+      </c>
+      <c r="J17">
+        <f>SUM(J18:J19)</f>
+        <v/>
+      </c>
+      <c r="K17">
+        <f>SUM(K18:K19)</f>
+        <v/>
+      </c>
+      <c r="L17">
+        <f>SUM(L18:L19)</f>
+        <v/>
+      </c>
+      <c r="M17">
+        <f>SUM(M18:M19)</f>
+        <v/>
+      </c>
+      <c r="N17">
+        <f>SUM(B17:M17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>17051.47</v>
+      </c>
+      <c r="C18" t="n">
+        <v>18200.47</v>
+      </c>
+      <c r="D18" t="n">
+        <v>21530.13</v>
+      </c>
+      <c r="E18" t="n">
+        <v>24277.37</v>
+      </c>
+      <c r="F18" t="n">
+        <v>27127.32</v>
+      </c>
+      <c r="G18" t="n">
+        <v>25179.56</v>
+      </c>
+      <c r="N18">
+        <f>SUM(B18:M18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>64136.35</v>
+      </c>
+      <c r="C19" t="n">
+        <v>64388.71</v>
+      </c>
+      <c r="D19" t="n">
+        <v>54424.09</v>
+      </c>
+      <c r="E19" t="n">
+        <v>43319.58</v>
+      </c>
+      <c r="F19" t="n">
+        <v>43972.72</v>
+      </c>
+      <c r="G19" t="n">
+        <v>41227.21</v>
+      </c>
+      <c r="N19">
+        <f>SUM(B19:M19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>B18/B17</f>
+        <v/>
+      </c>
+      <c r="C20" s="19">
+        <f>C18/C17</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>D18/D17</f>
+        <v/>
+      </c>
+      <c r="E20" s="19">
+        <f>E18/E17</f>
+        <v/>
+      </c>
+      <c r="F20" s="19">
+        <f>F18/F17</f>
+        <v/>
+      </c>
+      <c r="G20" s="19">
+        <f>G18/G17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>26 Vs 25</t>
+        </is>
+      </c>
+      <c r="B21" s="20">
+        <f>(B17-B13)/B13</f>
+        <v/>
+      </c>
+      <c r="C21" s="20">
+        <f>(C17-C13)/C13</f>
+        <v/>
+      </c>
+      <c r="D21" s="20">
+        <f>(D17-D13)/D13</f>
+        <v/>
+      </c>
+      <c r="E21" s="20">
+        <f>(E17-E13)/E13</f>
+        <v/>
+      </c>
+      <c r="F21" s="20">
+        <f>(F17-F13)/F13</f>
+        <v/>
+      </c>
+      <c r="G21" s="20">
+        <f>(G17-G13)/G13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>Phuket — Revenue (M THB)</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E24" s="18" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F24" s="18" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G24" s="18" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H24" s="18" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I24" s="18" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J24" s="18" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K24" s="18" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L24" s="18" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M24" s="18" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N24" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B25">
+        <f>SUM(B26:B27)</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>SUM(C26:C27)</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>SUM(D26:D27)</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>SUM(E26:E27)</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>SUM(F26:F27)</f>
+        <v/>
+      </c>
+      <c r="G25">
+        <f>SUM(G26:G27)</f>
+        <v/>
+      </c>
+      <c r="H25">
+        <f>SUM(H26:H27)</f>
+        <v/>
+      </c>
+      <c r="I25">
+        <f>SUM(I26:I27)</f>
+        <v/>
+      </c>
+      <c r="J25">
+        <f>SUM(J26:J27)</f>
+        <v/>
+      </c>
+      <c r="K25">
+        <f>SUM(K26:K27)</f>
+        <v/>
+      </c>
+      <c r="L25">
+        <f>SUM(L26:L27)</f>
+        <v/>
+      </c>
+      <c r="M25">
+        <f>SUM(M26:M27)</f>
+        <v/>
+      </c>
+      <c r="N25">
+        <f>SUM(B25:M25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3170.01</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3192.57</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3360.38</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2662.25</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3198.5</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2856.93</v>
+      </c>
+      <c r="H26" t="n">
+        <v>4158.41</v>
+      </c>
+      <c r="I26" t="n">
+        <v>3303.29</v>
+      </c>
+      <c r="J26" t="n">
+        <v>3316.68</v>
+      </c>
+      <c r="K26" t="n">
+        <v>2772.87</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2375.54</v>
+      </c>
+      <c r="M26" t="n">
+        <v>2680.09</v>
+      </c>
+      <c r="N26">
+        <f>SUM(B26:M26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>31909.45</v>
+      </c>
+      <c r="C27" t="n">
+        <v>34281.2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>34822.13</v>
+      </c>
+      <c r="E27" t="n">
+        <v>37435.62</v>
+      </c>
+      <c r="F27" t="n">
+        <v>34799.15</v>
+      </c>
+      <c r="G27" t="n">
+        <v>34865.31</v>
+      </c>
+      <c r="H27" t="n">
+        <v>30834.2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>32170.66</v>
+      </c>
+      <c r="J27" t="n">
+        <v>31032.38</v>
+      </c>
+      <c r="K27" t="n">
+        <v>31263.75</v>
+      </c>
+      <c r="L27" t="n">
+        <v>35973.35</v>
+      </c>
+      <c r="M27" t="n">
+        <v>40263.46</v>
+      </c>
+      <c r="N27">
+        <f>SUM(B27:M27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B28" s="19">
+        <f>B26/B25</f>
+        <v/>
+      </c>
+      <c r="C28" s="19">
+        <f>C26/C25</f>
+        <v/>
+      </c>
+      <c r="D28" s="19">
+        <f>D26/D25</f>
+        <v/>
+      </c>
+      <c r="E28" s="19">
+        <f>E26/E25</f>
+        <v/>
+      </c>
+      <c r="F28" s="19">
+        <f>F26/F25</f>
+        <v/>
+      </c>
+      <c r="G28" s="19">
+        <f>G26/G25</f>
+        <v/>
+      </c>
+      <c r="H28" s="19">
+        <f>H26/H25</f>
+        <v/>
+      </c>
+      <c r="I28" s="19">
+        <f>I26/I25</f>
+        <v/>
+      </c>
+      <c r="J28" s="19">
+        <f>J26/J25</f>
+        <v/>
+      </c>
+      <c r="K28" s="19">
+        <f>K26/K25</f>
+        <v/>
+      </c>
+      <c r="L28" s="19">
+        <f>L26/L25</f>
+        <v/>
+      </c>
+      <c r="M28" s="19">
+        <f>M26/M25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B29">
+        <f>SUM(B30:B31)</f>
+        <v/>
+      </c>
+      <c r="C29">
+        <f>SUM(C30:C31)</f>
+        <v/>
+      </c>
+      <c r="D29">
+        <f>SUM(D30:D31)</f>
+        <v/>
+      </c>
+      <c r="E29">
+        <f>SUM(E30:E31)</f>
+        <v/>
+      </c>
+      <c r="F29">
+        <f>SUM(F30:F31)</f>
+        <v/>
+      </c>
+      <c r="G29">
+        <f>SUM(G30:G31)</f>
+        <v/>
+      </c>
+      <c r="H29">
+        <f>SUM(H30:H31)</f>
+        <v/>
+      </c>
+      <c r="I29">
+        <f>SUM(I30:I31)</f>
+        <v/>
+      </c>
+      <c r="J29">
+        <f>SUM(J30:J31)</f>
+        <v/>
+      </c>
+      <c r="K29">
+        <f>SUM(K30:K31)</f>
+        <v/>
+      </c>
+      <c r="L29">
+        <f>SUM(L30:L31)</f>
+        <v/>
+      </c>
+      <c r="M29">
+        <f>SUM(M30:M31)</f>
+        <v/>
+      </c>
+      <c r="N29">
+        <f>SUM(B29:M29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>2817.32</v>
+      </c>
+      <c r="C30" t="n">
+        <v>3341.5</v>
+      </c>
+      <c r="D30" t="n">
+        <v>3439.77</v>
+      </c>
+      <c r="E30" t="n">
+        <v>3389.21</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3197.3</v>
+      </c>
+      <c r="G30" t="n">
+        <v>3760.78</v>
+      </c>
+      <c r="H30" t="n">
+        <v>2729.67</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3492.08</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3289.08</v>
+      </c>
+      <c r="K30" t="n">
+        <v>2946.59</v>
+      </c>
+      <c r="L30" t="n">
+        <v>2925.56</v>
+      </c>
+      <c r="M30" t="n">
+        <v>3304</v>
+      </c>
+      <c r="N30">
+        <f>SUM(B30:M30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>44364.03</v>
+      </c>
+      <c r="C31" t="n">
+        <v>43334.19</v>
+      </c>
+      <c r="D31" t="n">
+        <v>39639.23</v>
+      </c>
+      <c r="E31" t="n">
+        <v>44017.93</v>
+      </c>
+      <c r="F31" t="n">
+        <v>41361.59</v>
+      </c>
+      <c r="G31" t="n">
+        <v>42040.26</v>
+      </c>
+      <c r="H31" t="n">
+        <v>46932.54</v>
+      </c>
+      <c r="I31" t="n">
+        <v>46619.93</v>
+      </c>
+      <c r="J31" t="n">
+        <v>44392.01</v>
+      </c>
+      <c r="K31" t="n">
+        <v>40421.6</v>
+      </c>
+      <c r="L31" t="n">
+        <v>48934.82</v>
+      </c>
+      <c r="M31" t="n">
+        <v>50859.01</v>
+      </c>
+      <c r="N31">
+        <f>SUM(B31:M31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B32" s="19">
+        <f>B30/B29</f>
+        <v/>
+      </c>
+      <c r="C32" s="19">
+        <f>C30/C29</f>
+        <v/>
+      </c>
+      <c r="D32" s="19">
+        <f>D30/D29</f>
+        <v/>
+      </c>
+      <c r="E32" s="19">
+        <f>E30/E29</f>
+        <v/>
+      </c>
+      <c r="F32" s="19">
+        <f>F30/F29</f>
+        <v/>
+      </c>
+      <c r="G32" s="19">
+        <f>G30/G29</f>
+        <v/>
+      </c>
+      <c r="H32" s="19">
+        <f>H30/H29</f>
+        <v/>
+      </c>
+      <c r="I32" s="19">
+        <f>I30/I29</f>
+        <v/>
+      </c>
+      <c r="J32" s="19">
+        <f>J30/J29</f>
+        <v/>
+      </c>
+      <c r="K32" s="19">
+        <f>K30/K29</f>
+        <v/>
+      </c>
+      <c r="L32" s="19">
+        <f>L30/L29</f>
+        <v/>
+      </c>
+      <c r="M32" s="19">
+        <f>M30/M29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="18" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B33">
+        <f>SUM(B34:B35)</f>
+        <v/>
+      </c>
+      <c r="C33">
+        <f>SUM(C34:C35)</f>
+        <v/>
+      </c>
+      <c r="D33">
+        <f>SUM(D34:D35)</f>
+        <v/>
+      </c>
+      <c r="E33">
+        <f>SUM(E34:E35)</f>
+        <v/>
+      </c>
+      <c r="F33">
+        <f>SUM(F34:F35)</f>
+        <v/>
+      </c>
+      <c r="G33">
+        <f>SUM(G34:G35)</f>
+        <v/>
+      </c>
+      <c r="H33">
+        <f>SUM(H34:H35)</f>
+        <v/>
+      </c>
+      <c r="I33">
+        <f>SUM(I34:I35)</f>
+        <v/>
+      </c>
+      <c r="J33">
+        <f>SUM(J34:J35)</f>
+        <v/>
+      </c>
+      <c r="K33">
+        <f>SUM(K34:K35)</f>
+        <v/>
+      </c>
+      <c r="L33">
+        <f>SUM(L34:L35)</f>
+        <v/>
+      </c>
+      <c r="M33">
+        <f>SUM(M34:M35)</f>
+        <v/>
+      </c>
+      <c r="N33">
+        <f>SUM(B33:M33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2558.73</v>
+      </c>
+      <c r="C34" t="n">
+        <v>3190.64</v>
+      </c>
+      <c r="D34" t="n">
+        <v>3442.14</v>
+      </c>
+      <c r="E34" t="n">
+        <v>3546.28</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3472.9</v>
+      </c>
+      <c r="G34" t="n">
+        <v>3699.41</v>
+      </c>
+      <c r="N34">
+        <f>SUM(B34:M34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>49559.4</v>
+      </c>
+      <c r="C35" t="n">
+        <v>43399.95</v>
+      </c>
+      <c r="D35" t="n">
+        <v>36941.83</v>
+      </c>
+      <c r="E35" t="n">
+        <v>41372.92</v>
+      </c>
+      <c r="F35" t="n">
+        <v>39022.7</v>
+      </c>
+      <c r="G35" t="n">
+        <v>34647.97</v>
+      </c>
+      <c r="N35">
+        <f>SUM(B35:M35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B36" s="19">
+        <f>B34/B33</f>
+        <v/>
+      </c>
+      <c r="C36" s="19">
+        <f>C34/C33</f>
+        <v/>
+      </c>
+      <c r="D36" s="19">
+        <f>D34/D33</f>
+        <v/>
+      </c>
+      <c r="E36" s="19">
+        <f>E34/E33</f>
+        <v/>
+      </c>
+      <c r="F36" s="19">
+        <f>F34/F33</f>
+        <v/>
+      </c>
+      <c r="G36" s="19">
+        <f>G34/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B37">
+        <f>SUM(B38:B39)</f>
+        <v/>
+      </c>
+      <c r="C37">
+        <f>SUM(C38:C39)</f>
+        <v/>
+      </c>
+      <c r="D37">
+        <f>SUM(D38:D39)</f>
+        <v/>
+      </c>
+      <c r="E37">
+        <f>SUM(E38:E39)</f>
+        <v/>
+      </c>
+      <c r="F37">
+        <f>SUM(F38:F39)</f>
+        <v/>
+      </c>
+      <c r="G37">
+        <f>SUM(G38:G39)</f>
+        <v/>
+      </c>
+      <c r="H37">
+        <f>SUM(H38:H39)</f>
+        <v/>
+      </c>
+      <c r="I37">
+        <f>SUM(I38:I39)</f>
+        <v/>
+      </c>
+      <c r="J37">
+        <f>SUM(J38:J39)</f>
+        <v/>
+      </c>
+      <c r="K37">
+        <f>SUM(K38:K39)</f>
+        <v/>
+      </c>
+      <c r="L37">
+        <f>SUM(L38:L39)</f>
+        <v/>
+      </c>
+      <c r="M37">
+        <f>SUM(M38:M39)</f>
+        <v/>
+      </c>
+      <c r="N37">
+        <f>SUM(B37:M37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>2801.91</v>
+      </c>
+      <c r="C38" t="n">
+        <v>3899.15</v>
+      </c>
+      <c r="D38" t="n">
+        <v>3492.74</v>
+      </c>
+      <c r="E38" t="n">
+        <v>3442.17</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3397.06</v>
+      </c>
+      <c r="G38" t="n">
+        <v>3531.71</v>
+      </c>
+      <c r="N38">
+        <f>SUM(B38:M38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>50004.81</v>
+      </c>
+      <c r="C39" t="n">
+        <v>44906.87</v>
+      </c>
+      <c r="D39" t="n">
+        <v>37564.06</v>
+      </c>
+      <c r="E39" t="n">
+        <v>39838.63</v>
+      </c>
+      <c r="F39" t="n">
+        <v>37994.31</v>
+      </c>
+      <c r="G39" t="n">
+        <v>32133.22</v>
+      </c>
+      <c r="N39">
+        <f>SUM(B39:M39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B40" s="19">
+        <f>B38/B37</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>C38/C37</f>
+        <v/>
+      </c>
+      <c r="D40" s="19">
+        <f>D38/D37</f>
+        <v/>
+      </c>
+      <c r="E40" s="19">
+        <f>E38/E37</f>
+        <v/>
+      </c>
+      <c r="F40" s="19">
+        <f>F38/F37</f>
+        <v/>
+      </c>
+      <c r="G40" s="19">
+        <f>G38/G37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>26 Vs 25</t>
+        </is>
+      </c>
+      <c r="B41" s="20">
+        <f>(B37-B33)/B33</f>
+        <v/>
+      </c>
+      <c r="C41" s="20">
+        <f>(C37-C33)/C33</f>
+        <v/>
+      </c>
+      <c r="D41" s="20">
+        <f>(D37-D33)/D33</f>
+        <v/>
+      </c>
+      <c r="E41" s="20">
+        <f>(E37-E33)/E33</f>
+        <v/>
+      </c>
+      <c r="F41" s="20">
+        <f>(F37-F33)/F33</f>
+        <v/>
+      </c>
+      <c r="G41" s="20">
+        <f>(G37-G33)/G33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Pattaya (Chonburi) — Revenue (M THB)</t>
+        </is>
+      </c>
+      <c r="B44" s="18" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="C44" s="18" t="inlineStr">
+        <is>
+          <t>Feb</t>
+        </is>
+      </c>
+      <c r="D44" s="18" t="inlineStr">
+        <is>
+          <t>Mar</t>
+        </is>
+      </c>
+      <c r="E44" s="18" t="inlineStr">
+        <is>
+          <t>Apr</t>
+        </is>
+      </c>
+      <c r="F44" s="18" t="inlineStr">
+        <is>
+          <t>May</t>
+        </is>
+      </c>
+      <c r="G44" s="18" t="inlineStr">
+        <is>
+          <t>Jun</t>
+        </is>
+      </c>
+      <c r="H44" s="18" t="inlineStr">
+        <is>
+          <t>Jul</t>
+        </is>
+      </c>
+      <c r="I44" s="18" t="inlineStr">
+        <is>
+          <t>Aug</t>
+        </is>
+      </c>
+      <c r="J44" s="18" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="K44" s="18" t="inlineStr">
+        <is>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="L44" s="18" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="M44" s="18" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="N44" s="18" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="18" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B45">
+        <f>SUM(B46:B47)</f>
+        <v/>
+      </c>
+      <c r="C45">
+        <f>SUM(C46:C47)</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>SUM(D46:D47)</f>
+        <v/>
+      </c>
+      <c r="E45">
+        <f>SUM(E46:E47)</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>SUM(F46:F47)</f>
+        <v/>
+      </c>
+      <c r="G45">
+        <f>SUM(G46:G47)</f>
+        <v/>
+      </c>
+      <c r="H45">
+        <f>SUM(H46:H47)</f>
+        <v/>
+      </c>
+      <c r="I45">
+        <f>SUM(I46:I47)</f>
+        <v/>
+      </c>
+      <c r="J45">
+        <f>SUM(J46:J47)</f>
+        <v/>
+      </c>
+      <c r="K45">
+        <f>SUM(K46:K47)</f>
+        <v/>
+      </c>
+      <c r="L45">
+        <f>SUM(L46:L47)</f>
+        <v/>
+      </c>
+      <c r="M45">
+        <f>SUM(M46:M47)</f>
+        <v/>
+      </c>
+      <c r="N45">
+        <f>SUM(B45:M45)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>7872.94</v>
+      </c>
+      <c r="C46" t="n">
+        <v>6213.61</v>
+      </c>
+      <c r="D46" t="n">
+        <v>6405.91</v>
+      </c>
+      <c r="E46" t="n">
+        <v>7278.19</v>
+      </c>
+      <c r="F46" t="n">
+        <v>7478.2</v>
+      </c>
+      <c r="G46" t="n">
+        <v>7392.38</v>
+      </c>
+      <c r="H46" t="n">
+        <v>5235.32</v>
+      </c>
+      <c r="I46" t="n">
+        <v>7579.15</v>
+      </c>
+      <c r="J46" t="n">
+        <v>5667.97</v>
+      </c>
+      <c r="K46" t="n">
+        <v>7974.47</v>
+      </c>
+      <c r="L46" t="n">
+        <v>9197.75</v>
+      </c>
+      <c r="M46" t="n">
+        <v>10307.82</v>
+      </c>
+      <c r="N46">
+        <f>SUM(B46:M46)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>15700.8</v>
+      </c>
+      <c r="C47" t="n">
+        <v>15743.81</v>
+      </c>
+      <c r="D47" t="n">
+        <v>17423.74</v>
+      </c>
+      <c r="E47" t="n">
+        <v>19323.18</v>
+      </c>
+      <c r="F47" t="n">
+        <v>18115.09</v>
+      </c>
+      <c r="G47" t="n">
+        <v>18953.68</v>
+      </c>
+      <c r="H47" t="n">
+        <v>18985.08</v>
+      </c>
+      <c r="I47" t="n">
+        <v>17793.56</v>
+      </c>
+      <c r="J47" t="n">
+        <v>17243.37</v>
+      </c>
+      <c r="K47" t="n">
+        <v>15304.05</v>
+      </c>
+      <c r="L47" t="n">
+        <v>16418.89</v>
+      </c>
+      <c r="M47" t="n">
+        <v>18362.22</v>
+      </c>
+      <c r="N47">
+        <f>SUM(B47:M47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B48" s="19">
+        <f>B46/B45</f>
+        <v/>
+      </c>
+      <c r="C48" s="19">
+        <f>C46/C45</f>
+        <v/>
+      </c>
+      <c r="D48" s="19">
+        <f>D46/D45</f>
+        <v/>
+      </c>
+      <c r="E48" s="19">
+        <f>E46/E45</f>
+        <v/>
+      </c>
+      <c r="F48" s="19">
+        <f>F46/F45</f>
+        <v/>
+      </c>
+      <c r="G48" s="19">
+        <f>G46/G45</f>
+        <v/>
+      </c>
+      <c r="H48" s="19">
+        <f>H46/H45</f>
+        <v/>
+      </c>
+      <c r="I48" s="19">
+        <f>I46/I45</f>
+        <v/>
+      </c>
+      <c r="J48" s="19">
+        <f>J46/J45</f>
+        <v/>
+      </c>
+      <c r="K48" s="19">
+        <f>K46/K45</f>
+        <v/>
+      </c>
+      <c r="L48" s="19">
+        <f>L46/L45</f>
+        <v/>
+      </c>
+      <c r="M48" s="19">
+        <f>M46/M45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="18" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B49">
+        <f>SUM(B50:B51)</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>SUM(C50:C51)</f>
+        <v/>
+      </c>
+      <c r="D49">
+        <f>SUM(D50:D51)</f>
+        <v/>
+      </c>
+      <c r="E49">
+        <f>SUM(E50:E51)</f>
+        <v/>
+      </c>
+      <c r="F49">
+        <f>SUM(F50:F51)</f>
+        <v/>
+      </c>
+      <c r="G49">
+        <f>SUM(G50:G51)</f>
+        <v/>
+      </c>
+      <c r="H49">
+        <f>SUM(H50:H51)</f>
+        <v/>
+      </c>
+      <c r="I49">
+        <f>SUM(I50:I51)</f>
+        <v/>
+      </c>
+      <c r="J49">
+        <f>SUM(J50:J51)</f>
+        <v/>
+      </c>
+      <c r="K49">
+        <f>SUM(K50:K51)</f>
+        <v/>
+      </c>
+      <c r="L49">
+        <f>SUM(L50:L51)</f>
+        <v/>
+      </c>
+      <c r="M49">
+        <f>SUM(M50:M51)</f>
+        <v/>
+      </c>
+      <c r="N49">
+        <f>SUM(B49:M49)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>7019.43</v>
+      </c>
+      <c r="C50" t="n">
+        <v>6371.26</v>
+      </c>
+      <c r="D50" t="n">
+        <v>7554.39</v>
+      </c>
+      <c r="E50" t="n">
+        <v>9319.559999999999</v>
+      </c>
+      <c r="F50" t="n">
+        <v>9440.73</v>
+      </c>
+      <c r="G50" t="n">
+        <v>8519.120000000001</v>
+      </c>
+      <c r="H50" t="n">
+        <v>7727.16</v>
+      </c>
+      <c r="I50" t="n">
+        <v>9040.52</v>
+      </c>
+      <c r="J50" t="n">
+        <v>8759.33</v>
+      </c>
+      <c r="K50" t="n">
+        <v>9175.889999999999</v>
+      </c>
+      <c r="L50" t="n">
+        <v>9982.35</v>
+      </c>
+      <c r="M50" t="n">
+        <v>10983.61</v>
+      </c>
+      <c r="N50">
+        <f>SUM(B50:M50)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>21912.47</v>
+      </c>
+      <c r="C51" t="n">
+        <v>23600.45</v>
+      </c>
+      <c r="D51" t="n">
+        <v>22510.74</v>
+      </c>
+      <c r="E51" t="n">
+        <v>22567.81</v>
+      </c>
+      <c r="F51" t="n">
+        <v>19155.94</v>
+      </c>
+      <c r="G51" t="n">
+        <v>16870.14</v>
+      </c>
+      <c r="H51" t="n">
+        <v>19984.79</v>
+      </c>
+      <c r="I51" t="n">
+        <v>17581.73</v>
+      </c>
+      <c r="J51" t="n">
+        <v>18200.77</v>
+      </c>
+      <c r="K51" t="n">
+        <v>18212.67</v>
+      </c>
+      <c r="L51" t="n">
+        <v>18781.89</v>
+      </c>
+      <c r="M51" t="n">
+        <v>20030.39</v>
+      </c>
+      <c r="N51">
+        <f>SUM(B51:M51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B52" s="19">
+        <f>B50/B49</f>
+        <v/>
+      </c>
+      <c r="C52" s="19">
+        <f>C50/C49</f>
+        <v/>
+      </c>
+      <c r="D52" s="19">
+        <f>D50/D49</f>
+        <v/>
+      </c>
+      <c r="E52" s="19">
+        <f>E50/E49</f>
+        <v/>
+      </c>
+      <c r="F52" s="19">
+        <f>F50/F49</f>
+        <v/>
+      </c>
+      <c r="G52" s="19">
+        <f>G50/G49</f>
+        <v/>
+      </c>
+      <c r="H52" s="19">
+        <f>H50/H49</f>
+        <v/>
+      </c>
+      <c r="I52" s="19">
+        <f>I50/I49</f>
+        <v/>
+      </c>
+      <c r="J52" s="19">
+        <f>J50/J49</f>
+        <v/>
+      </c>
+      <c r="K52" s="19">
+        <f>K50/K49</f>
+        <v/>
+      </c>
+      <c r="L52" s="19">
+        <f>L50/L49</f>
+        <v/>
+      </c>
+      <c r="M52" s="19">
+        <f>M50/M49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="18" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B53">
+        <f>SUM(B54:B55)</f>
+        <v/>
+      </c>
+      <c r="C53">
+        <f>SUM(C54:C55)</f>
+        <v/>
+      </c>
+      <c r="D53">
+        <f>SUM(D54:D55)</f>
+        <v/>
+      </c>
+      <c r="E53">
+        <f>SUM(E54:E55)</f>
+        <v/>
+      </c>
+      <c r="F53">
+        <f>SUM(F54:F55)</f>
+        <v/>
+      </c>
+      <c r="G53">
+        <f>SUM(G54:G55)</f>
+        <v/>
+      </c>
+      <c r="H53">
+        <f>SUM(H54:H55)</f>
+        <v/>
+      </c>
+      <c r="I53">
+        <f>SUM(I54:I55)</f>
+        <v/>
+      </c>
+      <c r="J53">
+        <f>SUM(J54:J55)</f>
+        <v/>
+      </c>
+      <c r="K53">
+        <f>SUM(K54:K55)</f>
+        <v/>
+      </c>
+      <c r="L53">
+        <f>SUM(L54:L55)</f>
+        <v/>
+      </c>
+      <c r="M53">
+        <f>SUM(M54:M55)</f>
+        <v/>
+      </c>
+      <c r="N53">
+        <f>SUM(B53:M53)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>7885.24</v>
+      </c>
+      <c r="C54" t="n">
+        <v>7864.34</v>
+      </c>
+      <c r="D54" t="n">
+        <v>9154.08</v>
+      </c>
+      <c r="E54" t="n">
+        <v>12119.08</v>
+      </c>
+      <c r="F54" t="n">
+        <v>11342.65</v>
+      </c>
+      <c r="G54" t="n">
+        <v>8878.83</v>
+      </c>
+      <c r="N54">
+        <f>SUM(B54:M54)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>23069.56</v>
+      </c>
+      <c r="C55" t="n">
+        <v>22080.37</v>
+      </c>
+      <c r="D55" t="n">
+        <v>22095</v>
+      </c>
+      <c r="E55" t="n">
+        <v>19112.72</v>
+      </c>
+      <c r="F55" t="n">
+        <v>16679.84</v>
+      </c>
+      <c r="G55" t="n">
+        <v>15501.51</v>
+      </c>
+      <c r="N55">
+        <f>SUM(B55:M55)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B56" s="19">
+        <f>B54/B53</f>
+        <v/>
+      </c>
+      <c r="C56" s="19">
+        <f>C54/C53</f>
+        <v/>
+      </c>
+      <c r="D56" s="19">
+        <f>D54/D53</f>
+        <v/>
+      </c>
+      <c r="E56" s="19">
+        <f>E54/E53</f>
+        <v/>
+      </c>
+      <c r="F56" s="19">
+        <f>F54/F53</f>
+        <v/>
+      </c>
+      <c r="G56" s="19">
+        <f>G54/G53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="18" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B57">
+        <f>SUM(B58:B59)</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>SUM(C58:C59)</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>SUM(D58:D59)</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>SUM(E58:E59)</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>SUM(F58:F59)</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>SUM(G58:G59)</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>SUM(H58:H59)</f>
+        <v/>
+      </c>
+      <c r="I57">
+        <f>SUM(I58:I59)</f>
+        <v/>
+      </c>
+      <c r="J57">
+        <f>SUM(J58:J59)</f>
+        <v/>
+      </c>
+      <c r="K57">
+        <f>SUM(K58:K59)</f>
+        <v/>
+      </c>
+      <c r="L57">
+        <f>SUM(L58:L59)</f>
+        <v/>
+      </c>
+      <c r="M57">
+        <f>SUM(M58:M59)</f>
+        <v/>
+      </c>
+      <c r="N57">
+        <f>SUM(B57:M57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>- Domestics</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>7922.19</v>
+      </c>
+      <c r="C58" t="n">
+        <v>7548.57</v>
+      </c>
+      <c r="D58" t="n">
+        <v>8608.43</v>
+      </c>
+      <c r="E58" t="n">
+        <v>12581.91</v>
+      </c>
+      <c r="F58" t="n">
+        <v>11105.26</v>
+      </c>
+      <c r="G58" t="n">
+        <v>9072.809999999999</v>
+      </c>
+      <c r="N58">
+        <f>SUM(B58:M58)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>- International</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>20704.9</v>
+      </c>
+      <c r="C59" t="n">
+        <v>23791.9</v>
+      </c>
+      <c r="D59" t="n">
+        <v>21492.52</v>
+      </c>
+      <c r="E59" t="n">
+        <v>15939.63</v>
+      </c>
+      <c r="F59" t="n">
+        <v>16910.78</v>
+      </c>
+      <c r="G59" t="n">
+        <v>14482.54</v>
+      </c>
+      <c r="N59">
+        <f>SUM(B59:M59)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>% Domestic</t>
+        </is>
+      </c>
+      <c r="B60" s="19">
+        <f>B58/B57</f>
+        <v/>
+      </c>
+      <c r="C60" s="19">
+        <f>C58/C57</f>
+        <v/>
+      </c>
+      <c r="D60" s="19">
+        <f>D58/D57</f>
+        <v/>
+      </c>
+      <c r="E60" s="19">
+        <f>E58/E57</f>
+        <v/>
+      </c>
+      <c r="F60" s="19">
+        <f>F58/F57</f>
+        <v/>
+      </c>
+      <c r="G60" s="19">
+        <f>G58/G57</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>26 Vs 25</t>
+        </is>
+      </c>
+      <c r="B61" s="20">
+        <f>(B57-B53)/B53</f>
+        <v/>
+      </c>
+      <c r="C61" s="20">
+        <f>(C57-C53)/C53</f>
+        <v/>
+      </c>
+      <c r="D61" s="20">
+        <f>(D57-D53)/D53</f>
+        <v/>
+      </c>
+      <c r="E61" s="20">
+        <f>(E57-E53)/E53</f>
+        <v/>
+      </c>
+      <c r="F61" s="20">
+        <f>(F57-F53)/F53</f>
+        <v/>
+      </c>
+      <c r="G61" s="20">
+        <f>(G57-G53)/G53</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>